<commit_message>
changed default ports and started building out the excel file's power query
</commit_message>
<xml_diff>
--- a/api/assets/mock_collection.xlsx
+++ b/api/assets/mock_collection.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1147,7 +1147,116 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Base Set</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Charizard</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>NM</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Holo</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>2</v>
+      </c>
+      <c r="H22" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Fossil</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Gengar</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>NM</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Holo</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Jungle</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Flareon</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>LP</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>